<commit_message>
distillIQ_topK_spirit: a brand named in the raw name is a hard rule; unknown brands get no look-alikes
A brand from the hard truth or the brand lists named in the raw name restricts the options to that brand
(no more 1800 Double Barrel for a Jack Daniels Double Barrel); a leading brand word that no list knows
returns no liquor options; accents are folded; options below 0.5% calibrated confidence are not shown.
Out-of-fold liquor top-1/top-5 79.3%/88.5%, 0 cross-brand options on 2,972 branded raw names.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/topk_evaluation.xlsx
+++ b/topk_evaluation.xlsx
@@ -465,16 +465,16 @@
         <v>15997</v>
       </c>
       <c r="C2" t="n">
-        <v>0.939676189285491</v>
+        <v>0.9461148965431019</v>
       </c>
       <c r="D2" t="n">
+        <v>0.9758704757141964</v>
+      </c>
+      <c r="E2" t="n">
         <v>0.9762455460398825</v>
       </c>
-      <c r="E2" t="n">
-        <v>0.9766831280865163</v>
-      </c>
       <c r="F2" t="n">
-        <v>0.9766831280865163</v>
+        <v>0.9762455460398825</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -490,16 +490,16 @@
         <v>5371</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7806739899460063</v>
+        <v>0.7803016198100913</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8555203872649414</v>
+        <v>0.8551480171290262</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8713461180413331</v>
+        <v>0.8706013777695029</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8668776764103518</v>
+        <v>0.8661329361385217</v>
       </c>
       <c r="G3" t="n">
         <v>0.897039657419475</v>
@@ -515,16 +515,16 @@
         <v>2956</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8362652232746955</v>
+        <v>0.8349120433017592</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9012178619756428</v>
+        <v>0.9015561569688768</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9144113667117727</v>
+        <v>0.9133964817320703</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9086603518267929</v>
+        <v>0.9076454668470907</v>
       </c>
       <c r="G4" t="n">
         <v>0.9292963464140731</v>
@@ -540,16 +540,16 @@
         <v>2902</v>
       </c>
       <c r="C5" t="n">
-        <v>0.850447966919366</v>
+        <v>0.8480358373535493</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9221226740179187</v>
+        <v>0.9200551343900758</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9314266023432116</v>
+        <v>0.930737422467264</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9290144727773949</v>
+        <v>0.9279807029634735</v>
       </c>
       <c r="G5" t="n">
         <v>0.9441764300482426</v>
@@ -565,16 +565,16 @@
         <v>2631</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7844925883694412</v>
+        <v>0.7829722538958571</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8491068034967693</v>
+        <v>0.846826301786393</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8582288103382745</v>
+        <v>0.85480805777271</v>
       </c>
       <c r="F6" t="n">
-        <v>0.855188141391106</v>
+        <v>0.8517673888255416</v>
       </c>
       <c r="G6" t="n">
         <v>0.8760927404028886</v>
@@ -590,16 +590,16 @@
         <v>1103</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8640072529465095</v>
+        <v>0.8631006346328196</v>
       </c>
       <c r="D7" t="n">
-        <v>0.914777878513146</v>
+        <v>0.9138712601994561</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9202175883952856</v>
+        <v>0.9193109700815957</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9202175883952856</v>
+        <v>0.9193109700815957</v>
       </c>
       <c r="G7" t="n">
         <v>0.9356300997280145</v>
@@ -618,13 +618,13 @@
         <v>0.7600446428571429</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8582589285714286</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="E8" t="n">
-        <v>0.8828125</v>
+        <v>0.8772321428571429</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8794642857142857</v>
+        <v>0.8738839285714286</v>
       </c>
       <c r="G8" t="n">
         <v>0.8917410714285714</v>
@@ -640,16 +640,16 @@
         <v>430</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7790697674418605</v>
+        <v>0.7813953488372093</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8488372093023255</v>
+        <v>0.8465116279069768</v>
       </c>
       <c r="E9" t="n">
-        <v>0.8720930232558139</v>
+        <v>0.8744186046511628</v>
       </c>
       <c r="F9" t="n">
-        <v>0.8674418604651163</v>
+        <v>0.8697674418604651</v>
       </c>
       <c r="G9" t="n">
         <v>0.8976744186046511</v>
@@ -665,16 +665,16 @@
         <v>247</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8825910931174089</v>
+        <v>0.8744939271255061</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9068825910931174</v>
+        <v>0.8987854251012146</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9109311740890689</v>
+        <v>0.902834008097166</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9109311740890689</v>
+        <v>0.902834008097166</v>
       </c>
       <c r="G10" t="n">
         <v>0.9109311740890689</v>
@@ -690,16 +690,16 @@
         <v>78</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7948717948717948</v>
+        <v>0.7692307692307693</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8461538461538461</v>
+        <v>0.8205128205128205</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8461538461538461</v>
+        <v>0.8205128205128205</v>
       </c>
       <c r="F11" t="n">
-        <v>0.8461538461538461</v>
+        <v>0.8205128205128205</v>
       </c>
       <c r="G11" t="n">
         <v>0.8461538461538461</v>
@@ -873,13 +873,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>487</v>
+        <v>527</v>
       </c>
       <c r="C2" t="n">
-        <v>0.135523613963039</v>
+        <v>0.1233396584440228</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3675564681724846</v>
+        <v>0.3377609108159393</v>
       </c>
     </row>
     <row r="3">
@@ -889,13 +889,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1131</v>
+        <v>1117</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3191865605658709</v>
+        <v>0.3258728737690242</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6091954022988506</v>
+        <v>0.6177260519247986</v>
       </c>
     </row>
     <row r="4">
@@ -905,13 +905,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1619</v>
+        <v>1638</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5027794935145151</v>
+        <v>0.5054945054945055</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7473749227918468</v>
+        <v>0.7533577533577533</v>
       </c>
     </row>
     <row r="5">
@@ -921,13 +921,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2324</v>
+        <v>2311</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6544750430292599</v>
+        <v>0.6533967979229771</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8201376936316696</v>
+        <v>0.8126352228472523</v>
       </c>
     </row>
     <row r="6">
@@ -937,13 +937,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11556</v>
+        <v>11524</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9373485635167879</v>
+        <v>0.9377820201318986</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9684146763586016</v>
+        <v>0.9685005206525512</v>
       </c>
     </row>
   </sheetData>
@@ -1018,22 +1018,22 @@
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E2" t="n">
         <v>0.9824359711311235</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7941812233452124</v>
+        <v>0.7930127942980663</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9578463307146963</v>
+        <v>0.9643609886951523</v>
       </c>
       <c r="H2" t="n">
         <v>0.02307647368113571</v>
       </c>
       <c r="I2" t="n">
-        <v>1.185756651595036</v>
+        <v>1.185565421244959</v>
       </c>
     </row>
     <row r="3">
@@ -1047,22 +1047,22 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E3" t="n">
         <v>0.9862681228843329</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7941812233452124</v>
+        <v>0.7930127942980663</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9578463307146963</v>
+        <v>0.9652551574375678</v>
       </c>
       <c r="H3" t="n">
         <v>0.02804229713150669</v>
       </c>
       <c r="I3" t="n">
-        <v>1.185189815746456</v>
+        <v>1.18513271070774</v>
       </c>
     </row>
     <row r="4">
@@ -1076,22 +1076,22 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E4" t="n">
         <v>0.9798173340997637</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7941812233452124</v>
+        <v>0.7930127942980663</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9578463307146963</v>
+        <v>0.9636584275403972</v>
       </c>
       <c r="H4" t="n">
         <v>0.02167435882456038</v>
       </c>
       <c r="I4" t="n">
-        <v>1.185148390507644</v>
+        <v>1.184851775984353</v>
       </c>
     </row>
     <row r="5">
@@ -1105,51 +1105,51 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E5" t="n">
         <v>0.9824359711311235</v>
       </c>
       <c r="F5" t="n">
-        <v>0.7953496523923584</v>
+        <v>0.794122801892855</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9526090566519767</v>
       </c>
       <c r="H5" t="n">
         <v>0.02307647368113571</v>
       </c>
       <c r="I5" t="n">
-        <v>1.183431436933139</v>
+        <v>1.183969132577701</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="B6" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="C6" t="n">
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9906750974005237</v>
+        <v>0.9862681228843329</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7941812233452124</v>
+        <v>0.794122801892855</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9579101999105831</v>
+        <v>0.9535032253943923</v>
       </c>
       <c r="H6" t="n">
-        <v>0.03692235788981714</v>
+        <v>0.02804229713150669</v>
       </c>
       <c r="I6" t="n">
-        <v>1.182962853004779</v>
+        <v>1.183536422040482</v>
       </c>
     </row>
     <row r="7">
@@ -1157,57 +1157,57 @@
         <v>0.7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="C7" t="n">
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9862681228843329</v>
+        <v>0.9798173340997637</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7953496523923584</v>
+        <v>0.794122801892855</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9519064954972217</v>
       </c>
       <c r="H7" t="n">
-        <v>0.02804229713150669</v>
+        <v>0.02167435882456038</v>
       </c>
       <c r="I7" t="n">
-        <v>1.182864601084558</v>
+        <v>1.183255487317095</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="B8" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="C8" t="n">
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9798173340997637</v>
+        <v>0.9906750974005237</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7953496523923584</v>
+        <v>0.7930127942980663</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9411764705882353</v>
+        <v>0.9665325413553043</v>
       </c>
       <c r="H8" t="n">
-        <v>0.02167435882456038</v>
+        <v>0.03692235788981714</v>
       </c>
       <c r="I8" t="n">
-        <v>1.182823175845747</v>
+        <v>1.183087775174341</v>
       </c>
     </row>
     <row r="9">
@@ -1221,22 +1221,22 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E9" t="n">
         <v>0.9729833301398736</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7941812233452124</v>
+        <v>0.7930127942980663</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9577824615188095</v>
+        <v>0.9619978284473398</v>
       </c>
       <c r="H9" t="n">
         <v>0.01957118653969738</v>
       </c>
       <c r="I9" t="n">
-        <v>1.182773394290748</v>
+        <v>1.182237270282881</v>
       </c>
     </row>
     <row r="10">
@@ -1250,22 +1250,22 @@
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E10" t="n">
         <v>0.9906750974005237</v>
       </c>
       <c r="F10" t="n">
-        <v>0.7953496523923584</v>
+        <v>0.794122801892855</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9412403397841221</v>
+        <v>0.9547806093121287</v>
       </c>
       <c r="H10" t="n">
         <v>0.03692235788981714</v>
       </c>
       <c r="I10" t="n">
-        <v>1.180637638342882</v>
+        <v>1.181491486507083</v>
       </c>
     </row>
     <row r="11">
@@ -1279,22 +1279,22 @@
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E11" t="n">
         <v>0.9729833301398736</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7953496523923584</v>
+        <v>0.794122801892855</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9411126013923484</v>
+        <v>0.9502458964041642</v>
       </c>
       <c r="H11" t="n">
         <v>0.01957118653969738</v>
       </c>
       <c r="I11" t="n">
-        <v>1.18044817962885</v>
+        <v>1.180640981615623</v>
       </c>
     </row>
     <row r="12">
@@ -1308,22 +1308,22 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E12" t="n">
         <v>0.9824359711311235</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7978033533913653</v>
+        <v>0.7965180814395045</v>
       </c>
       <c r="G12" t="n">
-        <v>0.9018969151178386</v>
+        <v>0.924251133678227</v>
       </c>
       <c r="H12" t="n">
         <v>0.02307647368113571</v>
       </c>
       <c r="I12" t="n">
-        <v>1.177907558762431</v>
+        <v>1.180074736063636</v>
       </c>
     </row>
     <row r="13">
@@ -1337,22 +1337,22 @@
         <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E13" t="n">
         <v>0.9862681228843329</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7978033533913653</v>
+        <v>0.7965180814395045</v>
       </c>
       <c r="G13" t="n">
-        <v>0.9018969151178386</v>
+        <v>0.9251453024206425</v>
       </c>
       <c r="H13" t="n">
         <v>0.02804229713150669</v>
       </c>
       <c r="I13" t="n">
-        <v>1.17734072291385</v>
+        <v>1.179642025526417</v>
       </c>
     </row>
     <row r="14">
@@ -1366,22 +1366,22 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E14" t="n">
         <v>0.9798173340997637</v>
       </c>
       <c r="F14" t="n">
-        <v>0.7978033533913653</v>
+        <v>0.7965180814395045</v>
       </c>
       <c r="G14" t="n">
-        <v>0.9018969151178386</v>
+        <v>0.9235485725234719</v>
       </c>
       <c r="H14" t="n">
         <v>0.02167435882456038</v>
       </c>
       <c r="I14" t="n">
-        <v>1.177299297675038</v>
+        <v>1.17936109080303</v>
       </c>
     </row>
     <row r="15">
@@ -1395,22 +1395,22 @@
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E15" t="n">
         <v>0.9906750974005237</v>
       </c>
       <c r="F15" t="n">
-        <v>0.7978033533913653</v>
+        <v>0.7965180814395045</v>
       </c>
       <c r="G15" t="n">
-        <v>0.9019607843137255</v>
+        <v>0.926422686338379</v>
       </c>
       <c r="H15" t="n">
         <v>0.03692235788981714</v>
       </c>
       <c r="I15" t="n">
-        <v>1.175113760172173</v>
+        <v>1.177597089993018</v>
       </c>
     </row>
     <row r="16">
@@ -1424,22 +1424,22 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>0.8865455395221126</v>
+        <v>0.8845592101419641</v>
       </c>
       <c r="E16" t="n">
         <v>0.9729833301398736</v>
       </c>
       <c r="F16" t="n">
-        <v>0.7978033533913653</v>
+        <v>0.7965180814395045</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9018330459219518</v>
+        <v>0.9218879734304145</v>
       </c>
       <c r="H16" t="n">
         <v>0.01957118653969738</v>
       </c>
       <c r="I16" t="n">
-        <v>1.174924301458142</v>
+        <v>1.176746585101558</v>
       </c>
     </row>
     <row r="17">
@@ -1453,22 +1453,22 @@
         <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>0.8863702751650406</v>
+        <v>0.8843255243325349</v>
       </c>
       <c r="E17" t="n">
         <v>0.9952098103084882</v>
       </c>
       <c r="F17" t="n">
-        <v>0.7941812233452124</v>
+        <v>0.7930127942980663</v>
       </c>
       <c r="G17" t="n">
-        <v>0.95797406910647</v>
+        <v>0.967362840901833</v>
       </c>
       <c r="H17" t="n">
         <v>0.06093357480866975</v>
       </c>
       <c r="I17" t="n">
-        <v>1.173146549200182</v>
+        <v>1.173357225196161</v>
       </c>
     </row>
     <row r="18">
@@ -1482,22 +1482,22 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.8863702751650406</v>
+        <v>0.8843255243325349</v>
       </c>
       <c r="E18" t="n">
         <v>0.9952098103084882</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7953496523923584</v>
+        <v>0.794122801892855</v>
       </c>
       <c r="G18" t="n">
-        <v>0.941304208980009</v>
+        <v>0.9556109088586575</v>
       </c>
       <c r="H18" t="n">
         <v>0.06093357480866975</v>
       </c>
       <c r="I18" t="n">
-        <v>1.170821334538285</v>
+        <v>1.171760936528903</v>
       </c>
     </row>
     <row r="19">
@@ -1511,22 +1511,22 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>0.8863702751650406</v>
+        <v>0.8843255243325349</v>
       </c>
       <c r="E19" t="n">
         <v>0.9952098103084882</v>
       </c>
       <c r="F19" t="n">
-        <v>0.7978033533913653</v>
+        <v>0.7965180814395045</v>
       </c>
       <c r="G19" t="n">
-        <v>0.9020246535096124</v>
+        <v>0.9272529858849077</v>
       </c>
       <c r="H19" t="n">
         <v>0.06093357480866975</v>
       </c>
       <c r="I19" t="n">
-        <v>1.165297456367576</v>
+        <v>1.167866540014838</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
One spelling per product: repair broken encodings and fold accents (Anejo = Anejo); topK default brand zip, own .gitignore
textfix.py decodes UTF-8-as-cp1252 / GBK mojibake, restores lost letters from the known words and folds accents; used for
the hard truth at build time, for topK queries and for the tagger API (raw text in the output is untouched). Fixes
'1800 Tequila Anejo' being skipped by the tagger API. topK re-measured out-of-fold (liquor top-1/top-5 78.6%/87.8%).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/topk_evaluation.xlsx
+++ b/topk_evaluation.xlsx
@@ -462,19 +462,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15997</v>
+        <v>15993</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9461148965431019</v>
+        <v>0.9483524041768273</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9758704757141964</v>
+        <v>0.9793034452573001</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9762455460398825</v>
+        <v>0.9799912461701995</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9762455460398825</v>
+        <v>0.9799912461701995</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -490,19 +490,19 @@
         <v>5371</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7803016198100913</v>
+        <v>0.7767641035188978</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8551480171290262</v>
+        <v>0.8508657605660026</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8706013777695029</v>
+        <v>0.8681809718860547</v>
       </c>
       <c r="F3" t="n">
-        <v>0.8661329361385217</v>
+        <v>0.8629677899832433</v>
       </c>
       <c r="G3" t="n">
-        <v>0.897039657419475</v>
+        <v>0.8942468814001117</v>
       </c>
     </row>
     <row r="4">
@@ -515,19 +515,19 @@
         <v>2956</v>
       </c>
       <c r="C4" t="n">
-        <v>0.8349120433017592</v>
+        <v>0.8240866035182679</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9015561569688768</v>
+        <v>0.892083897158322</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9133964817320703</v>
+        <v>0.9035859269282814</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9076454668470907</v>
+        <v>0.8964817320703654</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9292963464140731</v>
+        <v>0.9211772665764547</v>
       </c>
     </row>
     <row r="5">
@@ -540,19 +540,19 @@
         <v>2902</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8480358373535493</v>
+        <v>0.8373535492763611</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9200551343900758</v>
+        <v>0.9110957960027567</v>
       </c>
       <c r="E5" t="n">
-        <v>0.930737422467264</v>
+        <v>0.9210889042039972</v>
       </c>
       <c r="F5" t="n">
-        <v>0.9279807029634735</v>
+        <v>0.919710544452102</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9441764300482426</v>
+        <v>0.9365954514128187</v>
       </c>
     </row>
     <row r="6">
@@ -565,19 +565,19 @@
         <v>2631</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7829722538958571</v>
+        <v>0.765868491068035</v>
       </c>
       <c r="D6" t="n">
-        <v>0.846826301786393</v>
+        <v>0.8323831242873432</v>
       </c>
       <c r="E6" t="n">
-        <v>0.85480805777271</v>
+        <v>0.8392246294184721</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8517673888255416</v>
+        <v>0.8350437096161155</v>
       </c>
       <c r="G6" t="n">
-        <v>0.8760927404028886</v>
+        <v>0.8624097301406309</v>
       </c>
     </row>
     <row r="7">
@@ -590,19 +590,19 @@
         <v>1103</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8631006346328196</v>
+        <v>0.8594741613780599</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9138712601994561</v>
+        <v>0.9093381686310064</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9193109700815957</v>
+        <v>0.9120580235720761</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9193109700815957</v>
+        <v>0.9111514052583862</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9356300997280145</v>
+        <v>0.9301903898458749</v>
       </c>
     </row>
     <row r="8">
@@ -615,19 +615,19 @@
         <v>896</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7600446428571429</v>
+        <v>0.7767857142857143</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.8694196428571429</v>
       </c>
       <c r="E8" t="n">
-        <v>0.8772321428571429</v>
+        <v>0.8850446428571429</v>
       </c>
       <c r="F8" t="n">
-        <v>0.8738839285714286</v>
+        <v>0.8783482142857143</v>
       </c>
       <c r="G8" t="n">
-        <v>0.8917410714285714</v>
+        <v>0.90625</v>
       </c>
     </row>
     <row r="9">
@@ -640,19 +640,19 @@
         <v>430</v>
       </c>
       <c r="C9" t="n">
-        <v>0.7813953488372093</v>
+        <v>0.7395348837209302</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8465116279069768</v>
+        <v>0.8186046511627907</v>
       </c>
       <c r="E9" t="n">
-        <v>0.8744186046511628</v>
+        <v>0.8372093023255814</v>
       </c>
       <c r="F9" t="n">
-        <v>0.8697674418604651</v>
+        <v>0.827906976744186</v>
       </c>
       <c r="G9" t="n">
-        <v>0.8976744186046511</v>
+        <v>0.8651162790697674</v>
       </c>
     </row>
     <row r="10">
@@ -665,19 +665,19 @@
         <v>247</v>
       </c>
       <c r="C10" t="n">
+        <v>0.8542510121457489</v>
+      </c>
+      <c r="D10" t="n">
         <v>0.8744939271255061</v>
       </c>
-      <c r="D10" t="n">
-        <v>0.8987854251012146</v>
-      </c>
       <c r="E10" t="n">
-        <v>0.902834008097166</v>
+        <v>0.8785425101214575</v>
       </c>
       <c r="F10" t="n">
-        <v>0.902834008097166</v>
+        <v>0.8785425101214575</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9109311740890689</v>
+        <v>0.8947368421052632</v>
       </c>
     </row>
     <row r="11">
@@ -690,19 +690,19 @@
         <v>78</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7692307692307693</v>
+        <v>0.782051282051282</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8205128205128205</v>
+        <v>0.8974358974358975</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8205128205128205</v>
+        <v>0.8974358974358975</v>
       </c>
       <c r="F11" t="n">
-        <v>0.8205128205128205</v>
+        <v>0.8974358974358975</v>
       </c>
       <c r="G11" t="n">
-        <v>0.8461538461538461</v>
+        <v>0.8974358974358975</v>
       </c>
     </row>
     <row r="12">
@@ -715,19 +715,19 @@
         <v>62</v>
       </c>
       <c r="C12" t="n">
-        <v>0.4193548387096774</v>
+        <v>0.532258064516129</v>
       </c>
       <c r="D12" t="n">
-        <v>0.4838709677419355</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="E12" t="n">
-        <v>0.4838709677419355</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="F12" t="n">
-        <v>0.4838709677419355</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="G12" t="n">
-        <v>0.4838709677419355</v>
+        <v>0.6129032258064516</v>
       </c>
     </row>
     <row r="13">
@@ -765,19 +765,19 @@
         <v>36</v>
       </c>
       <c r="C14" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E14" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F14" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="G14" t="n">
-        <v>0.8888888888888888</v>
+        <v>0.8333333333333334</v>
       </c>
     </row>
     <row r="15">
@@ -873,13 +873,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>527</v>
+        <v>559</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1233396584440228</v>
+        <v>0.1341681574239714</v>
       </c>
       <c r="D2" t="n">
-        <v>0.3377609108159393</v>
+        <v>0.3398926654740608</v>
       </c>
     </row>
     <row r="3">
@@ -889,13 +889,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1117</v>
+        <v>1143</v>
       </c>
       <c r="C3" t="n">
-        <v>0.3258728737690242</v>
+        <v>0.3079615048118985</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6177260519247986</v>
+        <v>0.5914260717410323</v>
       </c>
     </row>
     <row r="4">
@@ -905,13 +905,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1638</v>
+        <v>1582</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5054945054945055</v>
+        <v>0.4848293299620733</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7533577533577533</v>
+        <v>0.7402022756005057</v>
       </c>
     </row>
     <row r="5">
@@ -921,13 +921,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2311</v>
+        <v>2386</v>
       </c>
       <c r="C5" t="n">
-        <v>0.6533967979229771</v>
+        <v>0.6517183570829841</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8126352228472523</v>
+        <v>0.8164291701592624</v>
       </c>
     </row>
     <row r="6">
@@ -937,13 +937,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>11524</v>
+        <v>11444</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9377820201318986</v>
+        <v>0.9345508563439356</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9685005206525512</v>
+        <v>0.9642607479902132</v>
       </c>
     </row>
   </sheetData>
@@ -1012,28 +1012,28 @@
         <v>0.5</v>
       </c>
       <c r="B2" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="C2" t="n">
         <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.877644034124109</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9824359711311235</v>
+        <v>0.9860117526826776</v>
       </c>
       <c r="F2" t="n">
-        <v>0.7930127942980663</v>
+        <v>0.785555685403763</v>
       </c>
       <c r="G2" t="n">
-        <v>0.9643609886951523</v>
+        <v>0.9662749105774144</v>
       </c>
       <c r="H2" t="n">
-        <v>0.02307647368113571</v>
+        <v>0.02711230571461961</v>
       </c>
       <c r="I2" t="n">
-        <v>1.185565421244959</v>
+        <v>1.18104632994326</v>
       </c>
     </row>
     <row r="3">
@@ -1041,28 +1041,28 @@
         <v>0.5</v>
       </c>
       <c r="B3" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="C3" t="n">
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8777024658174594</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9862681228843329</v>
+        <v>0.9824987225344916</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7930127942980663</v>
+        <v>0.785555685403763</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9652551574375678</v>
+        <v>0.9653168114460909</v>
       </c>
       <c r="H3" t="n">
-        <v>0.02804229713150669</v>
+        <v>0.02343110903353979</v>
       </c>
       <c r="I3" t="n">
-        <v>1.18513271070774</v>
+        <v>1.181015914186684</v>
       </c>
     </row>
     <row r="4">
@@ -1076,22 +1076,22 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8777024658174594</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9798173340997637</v>
+        <v>0.9789218191108841</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7930127942980663</v>
+        <v>0.785555685403763</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9636584275403972</v>
+        <v>0.9646142054164537</v>
       </c>
       <c r="H4" t="n">
-        <v>0.02167435882456038</v>
+        <v>0.02150286315297417</v>
       </c>
       <c r="I4" t="n">
-        <v>1.184851775984353</v>
+        <v>1.180086194510717</v>
       </c>
     </row>
     <row r="5">
@@ -1099,28 +1099,28 @@
         <v>0.7</v>
       </c>
       <c r="B5" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="C5" t="n">
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.877644034124109</v>
       </c>
       <c r="E5" t="n">
-        <v>0.9824359711311235</v>
+        <v>0.9860117526826776</v>
       </c>
       <c r="F5" t="n">
-        <v>0.794122801892855</v>
+        <v>0.7864321608040201</v>
       </c>
       <c r="G5" t="n">
-        <v>0.9526090566519767</v>
+        <v>0.9532447623914154</v>
       </c>
       <c r="H5" t="n">
-        <v>0.02307647368113571</v>
+        <v>0.02711230571461961</v>
       </c>
       <c r="I5" t="n">
-        <v>1.183969132577701</v>
+        <v>1.179223279025399</v>
       </c>
     </row>
     <row r="6">
@@ -1128,86 +1128,86 @@
         <v>0.7</v>
       </c>
       <c r="B6" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="C6" t="n">
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8777024658174594</v>
       </c>
       <c r="E6" t="n">
-        <v>0.9862681228843329</v>
+        <v>0.9824987225344916</v>
       </c>
       <c r="F6" t="n">
-        <v>0.794122801892855</v>
+        <v>0.7864321608040201</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9535032253943923</v>
+        <v>0.9522866632600919</v>
       </c>
       <c r="H6" t="n">
-        <v>0.02804229713150669</v>
+        <v>0.02343110903353979</v>
       </c>
       <c r="I6" t="n">
-        <v>1.183536422040482</v>
+        <v>1.179192863268822</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="B7" t="n">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="C7" t="n">
         <v>2</v>
       </c>
       <c r="D7" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8775271707374079</v>
       </c>
       <c r="E7" t="n">
-        <v>0.9798173340997637</v>
+        <v>0.9902273888605008</v>
       </c>
       <c r="F7" t="n">
-        <v>0.794122801892855</v>
+        <v>0.785555685403763</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9519064954972217</v>
+        <v>0.9671691364333163</v>
       </c>
       <c r="H7" t="n">
-        <v>0.02167435882456038</v>
+        <v>0.03646137665069533</v>
       </c>
       <c r="I7" t="n">
-        <v>1.183255487317095</v>
+        <v>1.178555314749169</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="B8" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="C8" t="n">
         <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8777024658174594</v>
       </c>
       <c r="E8" t="n">
-        <v>0.9906750974005237</v>
+        <v>0.9789218191108841</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7930127942980663</v>
+        <v>0.7864321608040201</v>
       </c>
       <c r="G8" t="n">
-        <v>0.9665325413553043</v>
+        <v>0.9515840572304548</v>
       </c>
       <c r="H8" t="n">
-        <v>0.03692235788981714</v>
+        <v>0.02150286315297417</v>
       </c>
       <c r="I8" t="n">
-        <v>1.183087775174341</v>
+        <v>1.178263143592856</v>
       </c>
     </row>
     <row r="9">
@@ -1221,22 +1221,22 @@
         <v>2</v>
       </c>
       <c r="D9" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8777024658174594</v>
       </c>
       <c r="E9" t="n">
-        <v>0.9729833301398736</v>
+        <v>0.971895758814512</v>
       </c>
       <c r="F9" t="n">
-        <v>0.7930127942980663</v>
+        <v>0.785555685403763</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9619978284473398</v>
+        <v>0.9627618804292284</v>
       </c>
       <c r="H9" t="n">
-        <v>0.01957118653969738</v>
+        <v>0.01951618557905808</v>
       </c>
       <c r="I9" t="n">
-        <v>1.182237270282881</v>
+        <v>1.177288654401405</v>
       </c>
     </row>
     <row r="10">
@@ -1250,51 +1250,51 @@
         <v>2</v>
       </c>
       <c r="D10" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8775271707374079</v>
       </c>
       <c r="E10" t="n">
-        <v>0.9906750974005237</v>
+        <v>0.9902273888605008</v>
       </c>
       <c r="F10" t="n">
-        <v>0.794122801892855</v>
+        <v>0.7864321608040201</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9547806093121287</v>
+        <v>0.9541389882473174</v>
       </c>
       <c r="H10" t="n">
-        <v>0.03692235788981714</v>
+        <v>0.03646137665069533</v>
       </c>
       <c r="I10" t="n">
-        <v>1.181491486507083</v>
+        <v>1.176732263831307</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="B11" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="C11" t="n">
         <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.877644034124109</v>
       </c>
       <c r="E11" t="n">
-        <v>0.9729833301398736</v>
+        <v>0.9860117526826776</v>
       </c>
       <c r="F11" t="n">
-        <v>0.794122801892855</v>
+        <v>0.7891200186981419</v>
       </c>
       <c r="G11" t="n">
-        <v>0.9502458964041642</v>
+        <v>0.9264179867143587</v>
       </c>
       <c r="H11" t="n">
-        <v>0.01957118653969738</v>
+        <v>0.02711230571461961</v>
       </c>
       <c r="I11" t="n">
-        <v>1.180640981615623</v>
+        <v>1.175602441357958</v>
       </c>
     </row>
     <row r="12">
@@ -1308,51 +1308,51 @@
         <v>2</v>
       </c>
       <c r="D12" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8777024658174594</v>
       </c>
       <c r="E12" t="n">
-        <v>0.9824359711311235</v>
+        <v>0.9824987225344916</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7965180814395045</v>
+        <v>0.7891200186981419</v>
       </c>
       <c r="G12" t="n">
-        <v>0.924251133678227</v>
+        <v>0.9254598875830352</v>
       </c>
       <c r="H12" t="n">
-        <v>0.02307647368113571</v>
+        <v>0.02343110903353979</v>
       </c>
       <c r="I12" t="n">
-        <v>1.180074736063636</v>
+        <v>1.175572025601382</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="B13" t="n">
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="C13" t="n">
         <v>2</v>
       </c>
       <c r="D13" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8777024658174594</v>
       </c>
       <c r="E13" t="n">
-        <v>0.9862681228843329</v>
+        <v>0.971895758814512</v>
       </c>
       <c r="F13" t="n">
-        <v>0.7965180814395045</v>
+        <v>0.7864321608040201</v>
       </c>
       <c r="G13" t="n">
-        <v>0.9251453024206425</v>
+        <v>0.9497317322432295</v>
       </c>
       <c r="H13" t="n">
-        <v>0.02804229713150669</v>
+        <v>0.01951618557905808</v>
       </c>
       <c r="I13" t="n">
-        <v>1.179642025526417</v>
+        <v>1.175465603483544</v>
       </c>
     </row>
     <row r="14">
@@ -1366,22 +1366,22 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8777024658174594</v>
       </c>
       <c r="E14" t="n">
-        <v>0.9798173340997637</v>
+        <v>0.9789218191108841</v>
       </c>
       <c r="F14" t="n">
-        <v>0.7965180814395045</v>
+        <v>0.7891200186981419</v>
       </c>
       <c r="G14" t="n">
-        <v>0.9235485725234719</v>
+        <v>0.9247572815533981</v>
       </c>
       <c r="H14" t="n">
-        <v>0.02167435882456038</v>
+        <v>0.02150286315297417</v>
       </c>
       <c r="I14" t="n">
-        <v>1.17936109080303</v>
+        <v>1.174642305925415</v>
       </c>
     </row>
     <row r="15">
@@ -1395,22 +1395,22 @@
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8775271707374079</v>
       </c>
       <c r="E15" t="n">
-        <v>0.9906750974005237</v>
+        <v>0.9902273888605008</v>
       </c>
       <c r="F15" t="n">
-        <v>0.7965180814395045</v>
+        <v>0.7891200186981419</v>
       </c>
       <c r="G15" t="n">
-        <v>0.926422686338379</v>
+        <v>0.9273122125702606</v>
       </c>
       <c r="H15" t="n">
-        <v>0.03692235788981714</v>
+        <v>0.03646137665069533</v>
       </c>
       <c r="I15" t="n">
-        <v>1.177597089993018</v>
+        <v>1.173111426163867</v>
       </c>
     </row>
     <row r="16">
@@ -1424,22 +1424,22 @@
         <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>0.8845592101419641</v>
+        <v>0.8777024658174594</v>
       </c>
       <c r="E16" t="n">
-        <v>0.9729833301398736</v>
+        <v>0.971895758814512</v>
       </c>
       <c r="F16" t="n">
-        <v>0.7965180814395045</v>
+        <v>0.7891200186981419</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9218879734304145</v>
+        <v>0.9229049565661727</v>
       </c>
       <c r="H16" t="n">
-        <v>0.01957118653969738</v>
+        <v>0.01951618557905808</v>
       </c>
       <c r="I16" t="n">
-        <v>1.176746585101558</v>
+        <v>1.171844765816104</v>
       </c>
     </row>
     <row r="17">
@@ -1453,22 +1453,22 @@
         <v>2</v>
       </c>
       <c r="D17" t="n">
-        <v>0.8843255243325349</v>
+        <v>0.8772934439640061</v>
       </c>
       <c r="E17" t="n">
-        <v>0.9952098103084882</v>
+        <v>0.9949540112416965</v>
       </c>
       <c r="F17" t="n">
-        <v>0.7930127942980663</v>
+        <v>0.785555685403763</v>
       </c>
       <c r="G17" t="n">
-        <v>0.967362840901833</v>
+        <v>0.9682549821154829</v>
       </c>
       <c r="H17" t="n">
-        <v>0.06093357480866975</v>
+        <v>0.0599509173775856</v>
       </c>
       <c r="I17" t="n">
-        <v>1.173357225196161</v>
+        <v>1.169219869041945</v>
       </c>
     </row>
     <row r="18">
@@ -1482,22 +1482,22 @@
         <v>2</v>
       </c>
       <c r="D18" t="n">
-        <v>0.8843255243325349</v>
+        <v>0.8772934439640061</v>
       </c>
       <c r="E18" t="n">
-        <v>0.9952098103084882</v>
+        <v>0.9949540112416965</v>
       </c>
       <c r="F18" t="n">
-        <v>0.794122801892855</v>
+        <v>0.7864321608040201</v>
       </c>
       <c r="G18" t="n">
-        <v>0.9556109088586575</v>
+        <v>0.9552248339294839</v>
       </c>
       <c r="H18" t="n">
-        <v>0.06093357480866975</v>
+        <v>0.0599509173775856</v>
       </c>
       <c r="I18" t="n">
-        <v>1.171760936528903</v>
+        <v>1.167396818124084</v>
       </c>
     </row>
     <row r="19">
@@ -1511,22 +1511,22 @@
         <v>2</v>
       </c>
       <c r="D19" t="n">
-        <v>0.8843255243325349</v>
+        <v>0.8772934439640061</v>
       </c>
       <c r="E19" t="n">
-        <v>0.9952098103084882</v>
+        <v>0.9949540112416965</v>
       </c>
       <c r="F19" t="n">
-        <v>0.7965180814395045</v>
+        <v>0.7891200186981419</v>
       </c>
       <c r="G19" t="n">
-        <v>0.9272529858849077</v>
+        <v>0.9283980582524272</v>
       </c>
       <c r="H19" t="n">
-        <v>0.06093357480866975</v>
+        <v>0.0599509173775856</v>
       </c>
       <c r="I19" t="n">
-        <v>1.167866540014838</v>
+        <v>1.163775980456644</v>
       </c>
     </row>
   </sheetData>

</xml_diff>